<commit_message>
Precio mayorista configurable, fotos en cualquier formato
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014TUFyvu8kZ5oHv9NE5CpfU
</commit_message>
<xml_diff>
--- a/plantilla-catalogo.xlsx
+++ b/plantilla-catalogo.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:L3"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -405,10 +405,12 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" customWidth="1"/>
+    <col min="10" max="10" width="30.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -422,24 +424,30 @@
         <v>precio</v>
       </c>
       <c r="D1" t="str">
+        <v>precio_mayorista</v>
+      </c>
+      <c r="E1" t="str">
+        <v>minimo_mayorista</v>
+      </c>
+      <c r="F1" t="str">
         <v>precio_anterior</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>stock</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>variantes</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>descripcion</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>imagen</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>destacado</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>nuevo</v>
       </c>
     </row>
@@ -454,24 +462,30 @@
         <v>65000</v>
       </c>
       <c r="D2">
+        <v>55000</v>
+      </c>
+      <c r="E2">
+        <v>6</v>
+      </c>
+      <c r="F2">
         <v>80000</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>10</v>
       </c>
-      <c r="F2" t="str">
+      <c r="H2" t="str">
         <v>S, M, L</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>Algodón 100%</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>SI</v>
       </c>
-      <c r="J2" t="str">
+      <c r="L2" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -495,21 +509,27 @@
         <v/>
       </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
         <v>Talle único</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>https://…/foto.jpg</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
         <v>NO</v>
       </c>
-      <c r="J3" t="str">
+      <c r="L3" t="str">
         <v>SI</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>